<commit_message>
chore: refresh fixed 15-case payloads
</commit_message>
<xml_diff>
--- a/cases/longda_nscg_telework_hard/data/docs/TOGA_crosswalk_NSCG23_20250116.xlsx
+++ b/cases/longda_nscg_telework_hard/data/docs/TOGA_crosswalk_NSCG23_20250116.xlsx
@@ -4,7 +4,9 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15"/>
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Publication files\STI SM files\FY 2025\PUF - NSCG 2023\"/>
+    </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A036BF84-88D1-4EED-85E7-DB532113B7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>